<commit_message>
VisionQuest release dates updateds
</commit_message>
<xml_diff>
--- a/MCU.xlsx
+++ b/MCU.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\timeline-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A9D6E09-8898-4F49-A7A3-C08D2C94719B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76B3BB2B-6ADF-46A4-9DDF-A4D850303472}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -69866,7 +69866,7 @@
         <v>1218</v>
       </c>
       <c r="H1034" s="1">
-        <v>46316</v>
+        <v>46309</v>
       </c>
       <c r="K1034" t="s">
         <v>1282</v>
@@ -69907,7 +69907,7 @@
         <v>1222</v>
       </c>
       <c r="H1035" s="1">
-        <v>46323</v>
+        <v>46316</v>
       </c>
       <c r="K1035" t="s">
         <v>1282</v>
@@ -69948,7 +69948,7 @@
         <v>1225</v>
       </c>
       <c r="H1036" s="1">
-        <v>46330</v>
+        <v>46323</v>
       </c>
       <c r="K1036" t="s">
         <v>1282</v>
@@ -69989,7 +69989,7 @@
         <v>1228</v>
       </c>
       <c r="H1037" s="1">
-        <v>46337</v>
+        <v>46330</v>
       </c>
       <c r="K1037" t="s">
         <v>1282</v>
@@ -70030,7 +70030,7 @@
         <v>1232</v>
       </c>
       <c r="H1038" s="1">
-        <v>46344</v>
+        <v>46337</v>
       </c>
       <c r="K1038" t="s">
         <v>1282</v>
@@ -70071,7 +70071,7 @@
         <v>1236</v>
       </c>
       <c r="H1039" s="1">
-        <v>46351</v>
+        <v>46344</v>
       </c>
       <c r="K1039" t="s">
         <v>1282</v>
@@ -70112,7 +70112,7 @@
         <v>1240</v>
       </c>
       <c r="H1040" s="1">
-        <v>46358</v>
+        <v>46351</v>
       </c>
       <c r="K1040" t="s">
         <v>1282</v>

</xml_diff>

<commit_message>
Comma Error in universe labels
</commit_message>
<xml_diff>
--- a/MCU.xlsx
+++ b/MCU.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\timeline-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDC91499-2C25-4410-B197-D718118EEEB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC10F931-48CF-4885-A89B-BAD9CF40AB09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11917,10 +11917,10 @@
     <t>The Incredible Hulk (80s TV Show)</t>
   </si>
   <si>
-    <t>Marvel Animated Universe (Iron Man, Fantastic Four)</t>
-  </si>
-  <si>
-    <t>Marvel Animated Universe (X-Men, Spider-Man)</t>
+    <t>Marvel Animated Universe (X-Men &amp; Spider-Man)</t>
+  </si>
+  <si>
+    <t>Marvel Animated Universe (Iron Man &amp; Fantastic Four)</t>
   </si>
 </sst>
 </file>
@@ -20268,7 +20268,7 @@
         <v>386</v>
       </c>
       <c r="K155" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L155" t="s">
         <v>387</v>
@@ -20321,7 +20321,7 @@
         <v>386</v>
       </c>
       <c r="K156" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L156" t="s">
         <v>387</v>
@@ -20374,7 +20374,7 @@
         <v>386</v>
       </c>
       <c r="K157" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L157" t="s">
         <v>387</v>
@@ -20427,7 +20427,7 @@
         <v>400</v>
       </c>
       <c r="K158" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L158" t="s">
         <v>387</v>
@@ -20480,7 +20480,7 @@
         <v>400</v>
       </c>
       <c r="K159" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L159" t="s">
         <v>387</v>
@@ -20533,7 +20533,7 @@
         <v>400</v>
       </c>
       <c r="K160" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L160" t="s">
         <v>387</v>
@@ -20586,7 +20586,7 @@
         <v>400</v>
       </c>
       <c r="K161" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L161" t="s">
         <v>387</v>
@@ -20639,7 +20639,7 @@
         <v>400</v>
       </c>
       <c r="K162" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L162" t="s">
         <v>387</v>
@@ -20692,7 +20692,7 @@
         <v>416</v>
       </c>
       <c r="K163" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L163" t="s">
         <v>387</v>
@@ -20745,7 +20745,7 @@
         <v>420</v>
       </c>
       <c r="K164" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L164" t="s">
         <v>387</v>
@@ -20851,7 +20851,7 @@
         <v>425</v>
       </c>
       <c r="K166" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L166" t="s">
         <v>387</v>
@@ -20904,7 +20904,7 @@
         <v>425</v>
       </c>
       <c r="K167" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L167" t="s">
         <v>387</v>
@@ -21007,7 +21007,7 @@
         <v>434</v>
       </c>
       <c r="K169" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L169" t="s">
         <v>387</v>
@@ -21060,7 +21060,7 @@
         <v>438</v>
       </c>
       <c r="K170" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L170" t="s">
         <v>439</v>
@@ -21113,7 +21113,7 @@
         <v>438</v>
       </c>
       <c r="K171" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L171" t="s">
         <v>439</v>
@@ -21166,7 +21166,7 @@
         <v>438</v>
       </c>
       <c r="K172" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L172" t="s">
         <v>439</v>
@@ -21219,7 +21219,7 @@
         <v>438</v>
       </c>
       <c r="K173" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L173" t="s">
         <v>439</v>
@@ -21272,7 +21272,7 @@
         <v>453</v>
       </c>
       <c r="K174" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L174" t="s">
         <v>439</v>
@@ -21325,7 +21325,7 @@
         <v>453</v>
       </c>
       <c r="K175" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L175" t="s">
         <v>439</v>
@@ -21378,7 +21378,7 @@
         <v>453</v>
       </c>
       <c r="K176" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L176" t="s">
         <v>439</v>
@@ -21431,7 +21431,7 @@
         <v>453</v>
       </c>
       <c r="K177" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L177" t="s">
         <v>439</v>
@@ -21484,7 +21484,7 @@
         <v>453</v>
       </c>
       <c r="K178" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L178" t="s">
         <v>439</v>
@@ -21537,7 +21537,7 @@
         <v>453</v>
       </c>
       <c r="K179" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L179" t="s">
         <v>439</v>
@@ -21590,7 +21590,7 @@
         <v>453</v>
       </c>
       <c r="K180" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L180" t="s">
         <v>439</v>
@@ -21643,7 +21643,7 @@
         <v>475</v>
       </c>
       <c r="K181" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L181" t="s">
         <v>439</v>
@@ -21746,7 +21746,7 @@
         <v>521</v>
       </c>
       <c r="K183" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L183" t="s">
         <v>522</v>
@@ -21799,7 +21799,7 @@
         <v>514</v>
       </c>
       <c r="K184" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L184" t="s">
         <v>522</v>
@@ -21852,7 +21852,7 @@
         <v>514</v>
       </c>
       <c r="K185" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L185" t="s">
         <v>522</v>
@@ -21905,7 +21905,7 @@
         <v>514</v>
       </c>
       <c r="K186" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L186" t="s">
         <v>522</v>
@@ -21958,7 +21958,7 @@
         <v>514</v>
       </c>
       <c r="K187" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L187" t="s">
         <v>522</v>
@@ -22011,7 +22011,7 @@
         <v>514</v>
       </c>
       <c r="K188" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L188" t="s">
         <v>522</v>
@@ -22064,7 +22064,7 @@
         <v>514</v>
       </c>
       <c r="K189" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L189" t="s">
         <v>522</v>
@@ -22117,7 +22117,7 @@
         <v>514</v>
       </c>
       <c r="K190" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L190" t="s">
         <v>522</v>
@@ -22170,7 +22170,7 @@
         <v>514</v>
       </c>
       <c r="K191" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L191" t="s">
         <v>522</v>
@@ -22223,7 +22223,7 @@
         <v>514</v>
       </c>
       <c r="K192" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L192" t="s">
         <v>522</v>
@@ -22276,7 +22276,7 @@
         <v>514</v>
       </c>
       <c r="K193" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L193" t="s">
         <v>522</v>
@@ -22329,7 +22329,7 @@
         <v>514</v>
       </c>
       <c r="K194" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L194" t="s">
         <v>522</v>
@@ -22382,7 +22382,7 @@
         <v>514</v>
       </c>
       <c r="K195" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L195" t="s">
         <v>522</v>
@@ -22485,7 +22485,7 @@
         <v>514</v>
       </c>
       <c r="K197" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L197" t="s">
         <v>515</v>
@@ -22538,7 +22538,7 @@
         <v>514</v>
       </c>
       <c r="K198" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L198" t="s">
         <v>515</v>
@@ -22591,7 +22591,7 @@
         <v>514</v>
       </c>
       <c r="K199" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L199" t="s">
         <v>515</v>
@@ -22644,7 +22644,7 @@
         <v>514</v>
       </c>
       <c r="K200" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L200" t="s">
         <v>515</v>
@@ -22697,7 +22697,7 @@
         <v>514</v>
       </c>
       <c r="K201" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L201" t="s">
         <v>515</v>
@@ -22750,7 +22750,7 @@
         <v>514</v>
       </c>
       <c r="K202" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L202" t="s">
         <v>515</v>
@@ -22803,7 +22803,7 @@
         <v>514</v>
       </c>
       <c r="K203" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L203" t="s">
         <v>515</v>
@@ -22856,7 +22856,7 @@
         <v>514</v>
       </c>
       <c r="K204" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L204" t="s">
         <v>515</v>
@@ -22909,7 +22909,7 @@
         <v>514</v>
       </c>
       <c r="K205" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L205" t="s">
         <v>515</v>
@@ -22962,7 +22962,7 @@
         <v>514</v>
       </c>
       <c r="K206" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L206" t="s">
         <v>515</v>
@@ -23015,7 +23015,7 @@
         <v>514</v>
       </c>
       <c r="K207" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L207" t="s">
         <v>515</v>
@@ -23068,7 +23068,7 @@
         <v>514</v>
       </c>
       <c r="K208" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L208" t="s">
         <v>515</v>
@@ -23121,7 +23121,7 @@
         <v>514</v>
       </c>
       <c r="K209" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L209" t="s">
         <v>515</v>
@@ -23174,7 +23174,7 @@
         <v>581</v>
       </c>
       <c r="K210" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L210" t="s">
         <v>582</v>
@@ -23227,7 +23227,7 @@
         <v>623</v>
       </c>
       <c r="K211" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L211" t="s">
         <v>582</v>
@@ -23280,7 +23280,7 @@
         <v>479</v>
       </c>
       <c r="K212" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L212" t="s">
         <v>582</v>
@@ -23333,7 +23333,7 @@
         <v>479</v>
       </c>
       <c r="K213" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L213" t="s">
         <v>439</v>
@@ -23386,7 +23386,7 @@
         <v>479</v>
       </c>
       <c r="K214" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L214" t="s">
         <v>483</v>
@@ -23439,7 +23439,7 @@
         <v>479</v>
       </c>
       <c r="K215" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L215" t="s">
         <v>483</v>
@@ -23492,7 +23492,7 @@
         <v>479</v>
       </c>
       <c r="K216" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L216" t="s">
         <v>483</v>
@@ -23545,7 +23545,7 @@
         <v>479</v>
       </c>
       <c r="K217" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L217" t="s">
         <v>483</v>
@@ -23598,7 +23598,7 @@
         <v>479</v>
       </c>
       <c r="K218" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L218" t="s">
         <v>483</v>
@@ -23651,7 +23651,7 @@
         <v>479</v>
       </c>
       <c r="K219" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L219" t="s">
         <v>483</v>
@@ -23704,7 +23704,7 @@
         <v>479</v>
       </c>
       <c r="K220" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L220" t="s">
         <v>483</v>
@@ -23757,7 +23757,7 @@
         <v>527</v>
       </c>
       <c r="K221" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L221" t="s">
         <v>582</v>
@@ -23810,7 +23810,7 @@
         <v>527</v>
       </c>
       <c r="K222" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L222" t="s">
         <v>483</v>
@@ -23863,7 +23863,7 @@
         <v>527</v>
       </c>
       <c r="K223" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L223" t="s">
         <v>582</v>
@@ -23916,7 +23916,7 @@
         <v>527</v>
       </c>
       <c r="K224" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L224" t="s">
         <v>483</v>
@@ -23969,7 +23969,7 @@
         <v>527</v>
       </c>
       <c r="K225" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L225" t="s">
         <v>582</v>
@@ -24022,7 +24022,7 @@
         <v>527</v>
       </c>
       <c r="K226" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L226" t="s">
         <v>483</v>
@@ -24075,7 +24075,7 @@
         <v>527</v>
       </c>
       <c r="K227" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L227" t="s">
         <v>582</v>
@@ -24128,7 +24128,7 @@
         <v>627</v>
       </c>
       <c r="K228" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L228" t="s">
         <v>483</v>
@@ -24181,7 +24181,7 @@
         <v>627</v>
       </c>
       <c r="K229" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L229" t="s">
         <v>582</v>
@@ -24234,7 +24234,7 @@
         <v>627</v>
       </c>
       <c r="K230" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L230" t="s">
         <v>582</v>
@@ -24287,7 +24287,7 @@
         <v>627</v>
       </c>
       <c r="K231" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L231" t="s">
         <v>582</v>
@@ -24340,7 +24340,7 @@
         <v>667</v>
       </c>
       <c r="K232" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L232" t="s">
         <v>582</v>
@@ -24393,7 +24393,7 @@
         <v>671</v>
       </c>
       <c r="K233" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L233" t="s">
         <v>582</v>
@@ -24446,7 +24446,7 @@
         <v>671</v>
       </c>
       <c r="K234" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L234" t="s">
         <v>582</v>
@@ -24499,7 +24499,7 @@
         <v>697</v>
       </c>
       <c r="K235" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L235" t="s">
         <v>702</v>
@@ -24552,7 +24552,7 @@
         <v>697</v>
       </c>
       <c r="K236" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L236" t="s">
         <v>702</v>
@@ -24605,7 +24605,7 @@
         <v>697</v>
       </c>
       <c r="K237" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L237" t="s">
         <v>702</v>
@@ -24658,7 +24658,7 @@
         <v>697</v>
       </c>
       <c r="K238" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L238" t="s">
         <v>702</v>
@@ -24711,7 +24711,7 @@
         <v>697</v>
       </c>
       <c r="K239" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L239" t="s">
         <v>702</v>
@@ -24764,7 +24764,7 @@
         <v>697</v>
       </c>
       <c r="K240" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L240" t="s">
         <v>702</v>
@@ -24817,7 +24817,7 @@
         <v>697</v>
       </c>
       <c r="K241" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L241" t="s">
         <v>702</v>
@@ -24870,7 +24870,7 @@
         <v>697</v>
       </c>
       <c r="K242" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L242" t="s">
         <v>702</v>
@@ -24923,7 +24923,7 @@
         <v>697</v>
       </c>
       <c r="K243" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L243" t="s">
         <v>702</v>
@@ -24976,7 +24976,7 @@
         <v>697</v>
       </c>
       <c r="K244" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L244" t="s">
         <v>702</v>
@@ -25029,7 +25029,7 @@
         <v>697</v>
       </c>
       <c r="K245" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L245" t="s">
         <v>702</v>
@@ -25082,7 +25082,7 @@
         <v>697</v>
       </c>
       <c r="K246" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L246" t="s">
         <v>702</v>
@@ -25135,7 +25135,7 @@
         <v>697</v>
       </c>
       <c r="K247" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L247" t="s">
         <v>702</v>
@@ -25188,7 +25188,7 @@
         <v>697</v>
       </c>
       <c r="K248" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L248" t="s">
         <v>698</v>
@@ -25241,7 +25241,7 @@
         <v>697</v>
       </c>
       <c r="K249" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L249" t="s">
         <v>698</v>
@@ -25294,7 +25294,7 @@
         <v>697</v>
       </c>
       <c r="K250" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L250" t="s">
         <v>698</v>
@@ -25347,7 +25347,7 @@
         <v>697</v>
       </c>
       <c r="K251" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L251" t="s">
         <v>698</v>
@@ -25400,7 +25400,7 @@
         <v>697</v>
       </c>
       <c r="K252" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L252" t="s">
         <v>698</v>
@@ -25453,7 +25453,7 @@
         <v>697</v>
       </c>
       <c r="K253" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L253" t="s">
         <v>698</v>
@@ -25506,7 +25506,7 @@
         <v>697</v>
       </c>
       <c r="K254" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L254" t="s">
         <v>698</v>
@@ -25559,7 +25559,7 @@
         <v>697</v>
       </c>
       <c r="K255" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L255" t="s">
         <v>698</v>
@@ -25612,7 +25612,7 @@
         <v>697</v>
       </c>
       <c r="K256" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L256" t="s">
         <v>698</v>
@@ -25665,7 +25665,7 @@
         <v>506</v>
       </c>
       <c r="K257" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L257" t="s">
         <v>483</v>
@@ -25718,7 +25718,7 @@
         <v>506</v>
       </c>
       <c r="K258" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L258" t="s">
         <v>483</v>
@@ -25771,7 +25771,7 @@
         <v>573</v>
       </c>
       <c r="K259" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L259" t="s">
         <v>483</v>
@@ -25824,7 +25824,7 @@
         <v>573</v>
       </c>
       <c r="K260" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L260" t="s">
         <v>483</v>
@@ -25877,7 +25877,7 @@
         <v>573</v>
       </c>
       <c r="K261" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L261" t="s">
         <v>483</v>
@@ -25930,7 +25930,7 @@
         <v>573</v>
       </c>
       <c r="K262" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L262" t="s">
         <v>483</v>
@@ -25983,7 +25983,7 @@
         <v>573</v>
       </c>
       <c r="K263" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L263" t="s">
         <v>483</v>
@@ -26036,7 +26036,7 @@
         <v>573</v>
       </c>
       <c r="K264" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L264" t="s">
         <v>682</v>
@@ -26089,7 +26089,7 @@
         <v>573</v>
       </c>
       <c r="K265" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L265" t="s">
         <v>682</v>
@@ -26142,7 +26142,7 @@
         <v>573</v>
       </c>
       <c r="K266" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L266" t="s">
         <v>682</v>
@@ -26195,7 +26195,7 @@
         <v>573</v>
       </c>
       <c r="K267" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L267" t="s">
         <v>682</v>
@@ -26248,7 +26248,7 @@
         <v>573</v>
       </c>
       <c r="K268" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L268" t="s">
         <v>483</v>
@@ -26301,7 +26301,7 @@
         <v>573</v>
       </c>
       <c r="K269" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L269" t="s">
         <v>682</v>
@@ -26354,7 +26354,7 @@
         <v>573</v>
       </c>
       <c r="K270" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L270" t="s">
         <v>682</v>
@@ -26407,7 +26407,7 @@
         <v>573</v>
       </c>
       <c r="K271" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L271" t="s">
         <v>682</v>
@@ -26460,7 +26460,7 @@
         <v>573</v>
       </c>
       <c r="K272" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L272" t="s">
         <v>682</v>
@@ -26513,7 +26513,7 @@
         <v>573</v>
       </c>
       <c r="K273" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L273" t="s">
         <v>655</v>
@@ -26566,7 +26566,7 @@
         <v>573</v>
       </c>
       <c r="K274" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L274" t="s">
         <v>682</v>
@@ -26619,7 +26619,7 @@
         <v>573</v>
       </c>
       <c r="K275" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L275" t="s">
         <v>682</v>
@@ -26672,7 +26672,7 @@
         <v>823</v>
       </c>
       <c r="K276" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L276" t="s">
         <v>682</v>
@@ -26725,7 +26725,7 @@
         <v>823</v>
       </c>
       <c r="K277" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L277" t="s">
         <v>682</v>
@@ -26778,7 +26778,7 @@
         <v>823</v>
       </c>
       <c r="K278" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L278" t="s">
         <v>886</v>
@@ -26831,7 +26831,7 @@
         <v>823</v>
       </c>
       <c r="K279" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L279" t="s">
         <v>682</v>
@@ -26884,7 +26884,7 @@
         <v>823</v>
       </c>
       <c r="K280" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L280" t="s">
         <v>682</v>
@@ -26937,7 +26937,7 @@
         <v>823</v>
       </c>
       <c r="K281" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L281" t="s">
         <v>865</v>
@@ -26990,7 +26990,7 @@
         <v>751</v>
       </c>
       <c r="K282" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L282" t="s">
         <v>655</v>
@@ -27043,7 +27043,7 @@
         <v>751</v>
       </c>
       <c r="K283" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L283" t="s">
         <v>655</v>
@@ -27096,7 +27096,7 @@
         <v>710</v>
       </c>
       <c r="K284" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L284" t="s">
         <v>655</v>
@@ -27199,7 +27199,7 @@
         <v>710</v>
       </c>
       <c r="K286" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L286" t="s">
         <v>655</v>
@@ -27252,7 +27252,7 @@
         <v>852</v>
       </c>
       <c r="K287" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L287" t="s">
         <v>655</v>
@@ -27305,7 +27305,7 @@
         <v>852</v>
       </c>
       <c r="K288" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L288" t="s">
         <v>865</v>
@@ -27358,7 +27358,7 @@
         <v>663</v>
       </c>
       <c r="K289" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L289" t="s">
         <v>655</v>
@@ -27411,7 +27411,7 @@
         <v>687</v>
       </c>
       <c r="K290" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L290" t="s">
         <v>655</v>
@@ -27464,7 +27464,7 @@
         <v>687</v>
       </c>
       <c r="K291" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L291" t="s">
         <v>655</v>
@@ -27517,7 +27517,7 @@
         <v>714</v>
       </c>
       <c r="K292" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L292" t="s">
         <v>655</v>
@@ -27570,7 +27570,7 @@
         <v>714</v>
       </c>
       <c r="K293" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L293" t="s">
         <v>865</v>
@@ -27623,7 +27623,7 @@
         <v>714</v>
       </c>
       <c r="K294" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L294" t="s">
         <v>655</v>
@@ -27676,7 +27676,7 @@
         <v>714</v>
       </c>
       <c r="K295" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L295" t="s">
         <v>865</v>
@@ -27729,7 +27729,7 @@
         <v>714</v>
       </c>
       <c r="K296" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L296" t="s">
         <v>655</v>
@@ -27782,7 +27782,7 @@
         <v>714</v>
       </c>
       <c r="K297" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L297" t="s">
         <v>865</v>
@@ -27835,7 +27835,7 @@
         <v>714</v>
       </c>
       <c r="K298" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L298" t="s">
         <v>655</v>
@@ -27888,7 +27888,7 @@
         <v>827</v>
       </c>
       <c r="K299" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L299" t="s">
         <v>655</v>
@@ -27941,7 +27941,7 @@
         <v>678</v>
       </c>
       <c r="K300" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L300" t="s">
         <v>655</v>
@@ -27994,7 +27994,7 @@
         <v>678</v>
       </c>
       <c r="K301" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L301" t="s">
         <v>655</v>
@@ -28047,7 +28047,7 @@
         <v>771</v>
       </c>
       <c r="K302" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L302" t="s">
         <v>655</v>
@@ -28100,7 +28100,7 @@
         <v>771</v>
       </c>
       <c r="K303" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L303" t="s">
         <v>865</v>
@@ -28153,7 +28153,7 @@
         <v>771</v>
       </c>
       <c r="K304" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L304" t="s">
         <v>865</v>
@@ -28206,7 +28206,7 @@
         <v>771</v>
       </c>
       <c r="K305" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L305" t="s">
         <v>655</v>
@@ -28259,7 +28259,7 @@
         <v>771</v>
       </c>
       <c r="K306" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L306" t="s">
         <v>655</v>
@@ -28312,7 +28312,7 @@
         <v>771</v>
       </c>
       <c r="K307" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L307" t="s">
         <v>655</v>
@@ -28365,7 +28365,7 @@
         <v>885</v>
       </c>
       <c r="K308" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L308" t="s">
         <v>886</v>
@@ -28418,7 +28418,7 @@
         <v>885</v>
       </c>
       <c r="K309" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L309" t="s">
         <v>886</v>
@@ -28471,7 +28471,7 @@
         <v>885</v>
       </c>
       <c r="K310" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L310" t="s">
         <v>886</v>
@@ -28524,7 +28524,7 @@
         <v>885</v>
       </c>
       <c r="K311" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L311" t="s">
         <v>886</v>
@@ -28577,7 +28577,7 @@
         <v>923</v>
       </c>
       <c r="K312" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L312" t="s">
         <v>886</v>
@@ -28630,7 +28630,7 @@
         <v>923</v>
       </c>
       <c r="K313" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L313" t="s">
         <v>886</v>
@@ -28683,7 +28683,7 @@
         <v>923</v>
       </c>
       <c r="K314" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L314" t="s">
         <v>865</v>
@@ -28736,7 +28736,7 @@
         <v>933</v>
       </c>
       <c r="K315" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L315" t="s">
         <v>865</v>
@@ -28789,7 +28789,7 @@
         <v>937</v>
       </c>
       <c r="K316" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L316" t="s">
         <v>865</v>
@@ -28842,7 +28842,7 @@
         <v>937</v>
       </c>
       <c r="K317" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L317" t="s">
         <v>865</v>
@@ -28895,7 +28895,7 @@
         <v>937</v>
       </c>
       <c r="K318" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L318" t="s">
         <v>865</v>
@@ -28948,7 +28948,7 @@
         <v>965</v>
       </c>
       <c r="K319" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L319" t="s">
         <v>865</v>
@@ -29001,7 +29001,7 @@
         <v>965</v>
       </c>
       <c r="K320" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L320" t="s">
         <v>865</v>
@@ -29054,7 +29054,7 @@
         <v>965</v>
       </c>
       <c r="K321" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L321" t="s">
         <v>981</v>
@@ -29107,7 +29107,7 @@
         <v>989</v>
       </c>
       <c r="K322" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L322" t="s">
         <v>981</v>
@@ -29160,7 +29160,7 @@
         <v>989</v>
       </c>
       <c r="K323" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L323" t="s">
         <v>981</v>
@@ -29213,7 +29213,7 @@
         <v>989</v>
       </c>
       <c r="K324" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L324" t="s">
         <v>981</v>
@@ -29266,7 +29266,7 @@
         <v>989</v>
       </c>
       <c r="K325" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L325" t="s">
         <v>981</v>
@@ -29319,7 +29319,7 @@
         <v>891</v>
       </c>
       <c r="K326" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L326" t="s">
         <v>892</v>
@@ -29372,7 +29372,7 @@
         <v>891</v>
       </c>
       <c r="K327" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L327" t="s">
         <v>892</v>
@@ -29425,7 +29425,7 @@
         <v>891</v>
       </c>
       <c r="K328" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L328" t="s">
         <v>892</v>
@@ -29478,7 +29478,7 @@
         <v>891</v>
       </c>
       <c r="K329" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L329" t="s">
         <v>892</v>
@@ -29531,7 +29531,7 @@
         <v>891</v>
       </c>
       <c r="K330" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L330" t="s">
         <v>892</v>
@@ -29584,7 +29584,7 @@
         <v>891</v>
       </c>
       <c r="K331" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L331" t="s">
         <v>892</v>
@@ -29637,7 +29637,7 @@
         <v>891</v>
       </c>
       <c r="K332" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L332" t="s">
         <v>892</v>
@@ -29690,7 +29690,7 @@
         <v>891</v>
       </c>
       <c r="K333" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L333" t="s">
         <v>892</v>
@@ -29743,7 +29743,7 @@
         <v>891</v>
       </c>
       <c r="K334" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L334" t="s">
         <v>892</v>
@@ -29796,7 +29796,7 @@
         <v>891</v>
       </c>
       <c r="K335" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L335" t="s">
         <v>892</v>
@@ -29849,7 +29849,7 @@
         <v>891</v>
       </c>
       <c r="K336" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L336" t="s">
         <v>892</v>
@@ -29902,7 +29902,7 @@
         <v>891</v>
       </c>
       <c r="K337" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L337" t="s">
         <v>892</v>
@@ -29955,7 +29955,7 @@
         <v>891</v>
       </c>
       <c r="K338" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L338" t="s">
         <v>892</v>
@@ -30008,7 +30008,7 @@
         <v>1008</v>
       </c>
       <c r="K339" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L339" t="s">
         <v>981</v>
@@ -30061,7 +30061,7 @@
         <v>1008</v>
       </c>
       <c r="K340" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L340" t="s">
         <v>981</v>
@@ -30114,7 +30114,7 @@
         <v>1008</v>
       </c>
       <c r="K341" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L341" t="s">
         <v>886</v>
@@ -30167,7 +30167,7 @@
         <v>1008</v>
       </c>
       <c r="K342" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L342" t="s">
         <v>886</v>
@@ -30220,7 +30220,7 @@
         <v>1021</v>
       </c>
       <c r="K343" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L343" t="s">
         <v>981</v>
@@ -30273,7 +30273,7 @@
         <v>1021</v>
       </c>
       <c r="K344" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L344" t="s">
         <v>981</v>
@@ -30326,7 +30326,7 @@
         <v>1021</v>
       </c>
       <c r="K345" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L345" t="s">
         <v>981</v>
@@ -30379,7 +30379,7 @@
         <v>1031</v>
       </c>
       <c r="K346" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L346" t="s">
         <v>886</v>
@@ -30432,7 +30432,7 @@
         <v>1031</v>
       </c>
       <c r="K347" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L347" t="s">
         <v>886</v>
@@ -30485,7 +30485,7 @@
         <v>1031</v>
       </c>
       <c r="K348" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L348" t="s">
         <v>981</v>
@@ -30538,7 +30538,7 @@
         <v>1031</v>
       </c>
       <c r="K349" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L349" t="s">
         <v>1039</v>
@@ -30591,7 +30591,7 @@
         <v>1031</v>
       </c>
       <c r="K350" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L350" t="s">
         <v>1039</v>
@@ -30644,7 +30644,7 @@
         <v>1031</v>
       </c>
       <c r="K351" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L351" t="s">
         <v>1039</v>
@@ -30697,7 +30697,7 @@
         <v>1031</v>
       </c>
       <c r="K352" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L352" t="s">
         <v>1039</v>
@@ -30750,7 +30750,7 @@
         <v>1031</v>
       </c>
       <c r="K353" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L353" t="s">
         <v>1039</v>
@@ -30803,7 +30803,7 @@
         <v>1031</v>
       </c>
       <c r="K354" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L354" t="s">
         <v>1039</v>
@@ -30856,7 +30856,7 @@
         <v>1078</v>
       </c>
       <c r="K355" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L355" t="s">
         <v>1039</v>
@@ -30909,7 +30909,7 @@
         <v>1078</v>
       </c>
       <c r="K356" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L356" t="s">
         <v>1039</v>
@@ -30962,7 +30962,7 @@
         <v>1078</v>
       </c>
       <c r="K357" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L357" t="s">
         <v>1039</v>
@@ -31015,7 +31015,7 @@
         <v>1078</v>
       </c>
       <c r="K358" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L358" t="s">
         <v>1039</v>
@@ -31068,7 +31068,7 @@
         <v>1078</v>
       </c>
       <c r="K359" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L359" t="s">
         <v>1039</v>
@@ -31121,7 +31121,7 @@
         <v>1078</v>
       </c>
       <c r="K360" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L360" t="s">
         <v>1039</v>
@@ -31174,7 +31174,7 @@
         <v>1078</v>
       </c>
       <c r="K361" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L361" t="s">
         <v>1039</v>
@@ -31227,7 +31227,7 @@
         <v>761</v>
       </c>
       <c r="K362" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L362" t="s">
         <v>1055</v>
@@ -31280,7 +31280,7 @@
         <v>761</v>
       </c>
       <c r="K363" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L363" t="s">
         <v>1055</v>
@@ -31333,7 +31333,7 @@
         <v>761</v>
       </c>
       <c r="K364" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L364" t="s">
         <v>1055</v>
@@ -31386,7 +31386,7 @@
         <v>761</v>
       </c>
       <c r="K365" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L365" t="s">
         <v>1055</v>
@@ -31439,7 +31439,7 @@
         <v>761</v>
       </c>
       <c r="K366" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L366" t="s">
         <v>1055</v>
@@ -31492,7 +31492,7 @@
         <v>761</v>
       </c>
       <c r="K367" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L367" t="s">
         <v>1055</v>
@@ -31545,7 +31545,7 @@
         <v>761</v>
       </c>
       <c r="K368" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L368" t="s">
         <v>1055</v>
@@ -31598,7 +31598,7 @@
         <v>761</v>
       </c>
       <c r="K369" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L369" t="s">
         <v>1055</v>
@@ -31651,7 +31651,7 @@
         <v>761</v>
       </c>
       <c r="K370" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L370" t="s">
         <v>698</v>
@@ -31704,7 +31704,7 @@
         <v>761</v>
       </c>
       <c r="K371" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L371" t="s">
         <v>698</v>
@@ -31757,7 +31757,7 @@
         <v>761</v>
       </c>
       <c r="K372" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L372" t="s">
         <v>698</v>
@@ -31810,7 +31810,7 @@
         <v>761</v>
       </c>
       <c r="K373" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="L373" t="s">
         <v>698</v>
@@ -31863,7 +31863,7 @@
         <v>3468</v>
       </c>
       <c r="K374" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L374" t="s">
         <v>3469</v>
@@ -31916,7 +31916,7 @@
         <v>3468</v>
       </c>
       <c r="K375" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L375" t="s">
         <v>3469</v>
@@ -31969,7 +31969,7 @@
         <v>3468</v>
       </c>
       <c r="K376" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L376" t="s">
         <v>3469</v>
@@ -32022,7 +32022,7 @@
         <v>3468</v>
       </c>
       <c r="K377" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L377" t="s">
         <v>3469</v>
@@ -32075,7 +32075,7 @@
         <v>3483</v>
       </c>
       <c r="K378" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L378" t="s">
         <v>3469</v>
@@ -32128,7 +32128,7 @@
         <v>3483</v>
       </c>
       <c r="K379" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L379" t="s">
         <v>3469</v>
@@ -32181,7 +32181,7 @@
         <v>3483</v>
       </c>
       <c r="K380" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L380" t="s">
         <v>3469</v>
@@ -32234,7 +32234,7 @@
         <v>3493</v>
       </c>
       <c r="K381" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L381" t="s">
         <v>3469</v>
@@ -32287,7 +32287,7 @@
         <v>3493</v>
       </c>
       <c r="K382" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L382" t="s">
         <v>3469</v>
@@ -32340,7 +32340,7 @@
         <v>3500</v>
       </c>
       <c r="K383" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L383" t="s">
         <v>3469</v>
@@ -32393,7 +32393,7 @@
         <v>3500</v>
       </c>
       <c r="K384" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L384" t="s">
         <v>3815</v>
@@ -32446,7 +32446,7 @@
         <v>3942</v>
       </c>
       <c r="K385" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L385" t="s">
         <v>3815</v>
@@ -32493,7 +32493,7 @@
         <v>46204</v>
       </c>
       <c r="K386" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L386" t="s">
         <v>3815</v>
@@ -32540,7 +32540,7 @@
         <v>46211</v>
       </c>
       <c r="K387" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L387" t="s">
         <v>3815</v>
@@ -32587,7 +32587,7 @@
         <v>46218</v>
       </c>
       <c r="K388" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L388" t="s">
         <v>3815</v>
@@ -32640,7 +32640,7 @@
         <v>3941</v>
       </c>
       <c r="K389" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L389" t="s">
         <v>3815</v>
@@ -32693,7 +32693,7 @@
         <v>3940</v>
       </c>
       <c r="K390" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L390" t="s">
         <v>3815</v>
@@ -32746,7 +32746,7 @@
         <v>3940</v>
       </c>
       <c r="K391" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L391" t="s">
         <v>3815</v>
@@ -32799,7 +32799,7 @@
         <v>3940</v>
       </c>
       <c r="K392" t="s">
-        <v>3965</v>
+        <v>3964</v>
       </c>
       <c r="L392" t="s">
         <v>3815</v>

</xml_diff>

<commit_message>
X-men shared timeline data fix
</commit_message>
<xml_diff>
--- a/MCU.xlsx
+++ b/MCU.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\timeline-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC1FF041-26D1-4FD2-A620-6F7E3320F569}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A171086-992E-494F-9C1E-15E11D4BF70D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11920,10 +11920,10 @@
     <t>Marvel Animated Universe (Iron Man &amp; Fantastic Four)</t>
   </si>
   <si>
-    <t>Fox X-Men Erased Timeline (10005), Fox X-MenRevised Timeline (10005)</t>
-  </si>
-  <si>
     <t>Fox X-Men Revised Timeline (10005), Fox X-Men Erased Timeline (10005)</t>
+  </si>
+  <si>
+    <t>Fox X-Men Erased Timeline (10005), Fox X-Men Revised Timeline (10005)</t>
   </si>
 </sst>
 </file>
@@ -14446,7 +14446,7 @@
         <v>1301</v>
       </c>
       <c r="K40" t="s">
-        <v>3965</v>
+        <v>3966</v>
       </c>
       <c r="L40" t="s">
         <v>1302</v>
@@ -59053,7 +59053,7 @@
         <v>45106</v>
       </c>
       <c r="K889" t="s">
-        <v>3966</v>
+        <v>3965</v>
       </c>
       <c r="L889" t="s">
         <v>1477</v>

</xml_diff>

<commit_message>
VisionQuest Episode 5&6 Drop
</commit_message>
<xml_diff>
--- a/MCU.xlsx
+++ b/MCU.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\timeline-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A171086-992E-494F-9C1E-15E11D4BF70D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B87D1948-1518-475C-BF81-7001F59B95F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12454" uniqueCount="3967">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12458" uniqueCount="3967">
   <si>
     <t>id</t>
   </si>
@@ -66879,8 +66879,17 @@
       <c r="F1033" s="5" t="s">
         <v>3950</v>
       </c>
+      <c r="G1033">
+        <v>48</v>
+      </c>
       <c r="H1033" s="1">
         <v>46322</v>
+      </c>
+      <c r="I1033" s="3" t="s">
+        <v>3954</v>
+      </c>
+      <c r="J1033" s="3" t="s">
+        <v>3954</v>
       </c>
       <c r="K1033" t="s">
         <v>3956</v>
@@ -66923,8 +66932,17 @@
       <c r="F1034" s="5" t="s">
         <v>3951</v>
       </c>
+      <c r="G1034">
+        <v>57</v>
+      </c>
       <c r="H1034" s="1">
         <v>46322</v>
+      </c>
+      <c r="I1034" s="3" t="s">
+        <v>3954</v>
+      </c>
+      <c r="J1034" s="3" t="s">
+        <v>3954</v>
       </c>
       <c r="K1034" t="s">
         <v>3956</v>

</xml_diff>